<commit_message>
Fix Demand Forecast upload and remove hardcoded demo data
- Fix date parsing in forecast upload to support both yyyy/m/d and yyyy/mm/dd formats
- Handle Excel serial date numbers properly during upload
- Remove all hardcoded demo data from forecast_ctb_manager.js (user uploads only)
- Fix "Unsaved" badge showing incorrectly on page refresh in Production Plan config
- Add fallback logic to load demand data from localStorage in report generation
- Update repository documentation with server setup instructions

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Demo Summary/Forecast - v1.xlsx
+++ b/Demo Summary/Forecast - v1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chenhan/Documents/EDO/Demo Summary/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chenhan/Documents/FDOS/Demo Summary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5A61F45-39EA-534E-B108-08A4AECF7B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89AD248C-02C6-AE41-8D35-8CA7ADE3021A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15600" xr2:uid="{00D4898E-51D5-F44F-A983-48A11FF05C41}"/>
   </bookViews>
@@ -83,12 +83,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -432,49 +435,49 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2">
+      <c r="B1" s="3">
         <v>46291</v>
       </c>
-      <c r="C1" s="2">
+      <c r="C1" s="3">
         <v>46298</v>
       </c>
-      <c r="D1" s="2">
+      <c r="D1" s="3">
         <v>46305</v>
       </c>
-      <c r="E1" s="2">
+      <c r="E1" s="3">
         <v>46312</v>
       </c>
-      <c r="F1" s="2">
+      <c r="F1" s="3">
         <v>46319</v>
       </c>
-      <c r="G1" s="2">
+      <c r="G1" s="3">
         <v>46326</v>
       </c>
-      <c r="H1" s="2">
+      <c r="H1" s="3">
         <v>46333</v>
       </c>
-      <c r="I1" s="2">
+      <c r="I1" s="3">
         <v>46340</v>
       </c>
-      <c r="J1" s="2">
+      <c r="J1" s="3">
         <v>46347</v>
       </c>
-      <c r="K1" s="2">
+      <c r="K1" s="3">
         <v>46354</v>
       </c>
-      <c r="L1" s="2">
+      <c r="L1" s="3">
         <v>46361</v>
       </c>
-      <c r="M1" s="2">
+      <c r="M1" s="3">
         <v>46368</v>
       </c>
-      <c r="N1" s="2">
+      <c r="N1" s="3">
         <v>46375</v>
       </c>
-      <c r="O1" s="2">
+      <c r="O1" s="3">
         <v>46382</v>
       </c>
-      <c r="P1" s="2">
+      <c r="P1" s="3">
         <v>46389</v>
       </c>
       <c r="Q1" s="2"/>

</xml_diff>